<commit_message>
Apply style to cell
</commit_message>
<xml_diff>
--- a/internal/repository/testdata/Thu chi.xlsx
+++ b/internal/repository/testdata/Thu chi.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="47">
   <si>
     <t xml:space="preserve">CĂN TIN QUÁ KHỨ NĂM 2000</t>
   </si>
@@ -305,13 +305,16 @@
     <t xml:space="preserve">50000</t>
   </si>
   <si>
+    <t>SAMPLE TRANSACTION</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
     <t>2</t>
   </si>
   <si>
-    <t>Sample Transaction 2</t>
+    <t>SAMPLE TRANSACTION 2</t>
   </si>
   <si>
     <t>10</t>
@@ -324,13 +327,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ap="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:op="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing" xmlns:comp="http://schemas.openxmlformats.org/drawingml/2006/compatibility" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:lc="http://schemas.openxmlformats.org/drawingml/2006/lockedCanvas" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xne="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mso="http://schemas.microsoft.com/office/2006/01/customui" xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:cppr="http://schemas.microsoft.com/office/2006/coverPageProps" xmlns:cdip="http://schemas.microsoft.com/office/2006/customDocumentInformationPanel" xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ntns="http://schemas.microsoft.com/office/2006/metadata/customXsn" xmlns:lp="http://schemas.microsoft.com/office/2006/metadata/longProperties" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" xmlns:msink="http://schemas.microsoft.com/ink/2010/main" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" xmlns:cdr14="http://schemas.microsoft.com/office/drawing/2010/chartDrawing" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns:pic14="http://schemas.microsoft.com/office/drawing/2010/picture" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:dsp="http://schemas.microsoft.com/office/drawing/2008/diagram" xmlns:mso14="http://schemas.microsoft.com/office/2009/07/customui" xmlns:dgm14="http://schemas.microsoft.com/office/drawing/2010/diagram" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:xr4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision4" xmlns:xr5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision5" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr7="http://schemas.microsoft.com/office/spreadsheetml/2016/revision7" xmlns:xr8="http://schemas.microsoft.com/office/spreadsheetml/2016/revision8" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr11="http://schemas.microsoft.com/office/spreadsheetml/2016/revision11" xmlns:xr12="http://schemas.microsoft.com/office/spreadsheetml/2016/revision12" xmlns:xr13="http://schemas.microsoft.com/office/spreadsheetml/2016/revision13" xmlns:xr14="http://schemas.microsoft.com/office/spreadsheetml/2016/revision14" xmlns:xr15="http://schemas.microsoft.com/office/spreadsheetml/2016/revision15" xmlns:x16="http://schemas.microsoft.com/office/spreadsheetml/2014/11/main" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:mo="http://schemas.microsoft.com/office/mac/office/2008/main" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:v="urn:schemas-microsoft-com:vml" mc:Ignorable="c14 cdr14 a14 pic14 x14 xdr14 x14ac dsp mso14 dgm14 x15 x12ac x15ac xr xr2 xr3 xr4 xr5 xr6 xr7 xr8 xr9 xr10 xr11 xr12 xr13 xr14 xr15 x15 x16 x16r2 mo mx mv o v" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="m/d/yyyy"/>
     <numFmt numFmtId="166" formatCode="#,##0"/>
     <numFmt numFmtId="167" formatCode="0"/>
+    <numFmt numFmtId="168" formatCode="mm/dd/yyyy"/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="24">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -496,6 +500,13 @@
       <name val="Times New Roman"/>
       <family val="1"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
+      <color/>
+      <name val="Times New Roman"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="8">
@@ -542,7 +553,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -564,6 +575,21 @@
       <bottom style="thin"/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -590,7 +616,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="43">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom"/>
       <protection hidden="false" locked="true"/>
@@ -755,9 +781,11 @@
       <alignment horizontal="general" vertical="bottom"/>
       <protection hidden="false" locked="true"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="bottom"/>
-      <protection hidden="false" locked="true"/>
+    <xf numFmtId="168" fontId="23" fillId="0" borderId="3" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="false">
+      <alignment/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false">
+      <alignment/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -1730,20 +1758,75 @@
       <c r="L29" s="25"/>
       <c r="M29" s="31"/>
     </row>
-    <row r="30" ht="21">
-      <c r="B30" s="41" t="s">
-        <v>37</v>
-      </c>
-      <c r="C30" t="s">
-        <v>38</v>
-      </c>
-      <c r="D30" t="s">
-        <v>39</v>
-      </c>
-      <c r="K30" s="4" t="s">
-        <v>40</v>
-      </c>
-    </row>
+    <row r="1048329" ht="12.8"/>
+    <row r="1048330" ht="12.8"/>
+    <row r="1048331" ht="12.8"/>
+    <row r="1048332" ht="12.8"/>
+    <row r="1048333" ht="12.8"/>
+    <row r="1048334" ht="12.8"/>
+    <row r="1048335" ht="12.8"/>
+    <row r="1048336" ht="12.8"/>
+    <row r="1048337" ht="12.8"/>
+    <row r="1048338" ht="12.8"/>
+    <row r="1048339" ht="12.8"/>
+    <row r="1048340" ht="12.8"/>
+    <row r="1048341" ht="12.8"/>
+    <row r="1048342" ht="12.8"/>
+    <row r="1048343" ht="12.8"/>
+    <row r="1048344" ht="12.8"/>
+    <row r="1048345" ht="12.8"/>
+    <row r="1048346" ht="12.8"/>
+    <row r="1048347" ht="12.8"/>
+    <row r="1048348" ht="12.8"/>
+    <row r="1048349" ht="12.8"/>
+    <row r="1048350" ht="12.8"/>
+    <row r="1048351" ht="12.8"/>
+    <row r="1048352" ht="12.8"/>
+    <row r="1048353" ht="12.8"/>
+    <row r="1048354" ht="12.8"/>
+    <row r="1048355" ht="12.8"/>
+    <row r="1048356" ht="12.8"/>
+    <row r="1048357" ht="12.8"/>
+    <row r="1048358" ht="12.8"/>
+    <row r="1048359" ht="12.8"/>
+    <row r="1048360" ht="12.8"/>
+    <row r="1048361" ht="12.8"/>
+    <row r="1048362" ht="12.8"/>
+    <row r="1048363" ht="12.8"/>
+    <row r="1048364" ht="12.8"/>
+    <row r="1048365" ht="12.8"/>
+    <row r="1048366" ht="12.8"/>
+    <row r="1048367" ht="12.8"/>
+    <row r="1048368" ht="12.8"/>
+    <row r="1048369" ht="12.8"/>
+    <row r="1048370" ht="12.8"/>
+    <row r="1048371" ht="12.8"/>
+    <row r="1048372" ht="12.8"/>
+    <row r="1048373" ht="12.8"/>
+    <row r="1048374" ht="12.8"/>
+    <row r="1048375" ht="12.8"/>
+    <row r="1048376" ht="12.8"/>
+    <row r="1048377" ht="12.8"/>
+    <row r="1048378" ht="12.8"/>
+    <row r="1048379" ht="12.8"/>
+    <row r="1048380" ht="12.8"/>
+    <row r="1048381" ht="12.8"/>
+    <row r="1048382" ht="12.8"/>
+    <row r="1048383" ht="12.8"/>
+    <row r="1048384" ht="12.8"/>
+    <row r="1048385" ht="12.8"/>
+    <row r="1048386" ht="12.8"/>
+    <row r="1048387" ht="12.8"/>
+    <row r="1048388" ht="12.8"/>
+    <row r="1048389" ht="12.8"/>
+    <row r="1048390" ht="12.8"/>
+    <row r="1048391" ht="12.8"/>
+    <row r="1048392" ht="12.8"/>
+    <row r="1048393" ht="12.8"/>
+    <row r="1048394" ht="12.8"/>
+    <row r="1048395" ht="12.8"/>
+    <row r="1048396" ht="12.8"/>
+    <row r="1048397" ht="12.8"/>
     <row r="1048398" ht="12.8"/>
     <row r="1048399" ht="12.8"/>
     <row r="1048400" ht="12.8"/>
@@ -1833,75 +1916,63 @@
     <row r="1048484" ht="12.8"/>
     <row r="1048485" ht="12.8"/>
     <row r="1048486" ht="12.8"/>
-    <row r="1048487" ht="12.8"/>
-    <row r="1048488" ht="12.8"/>
-    <row r="1048489" ht="12.8"/>
-    <row r="1048490" ht="12.8"/>
-    <row r="1048491" ht="12.8"/>
-    <row r="1048492" ht="12.8"/>
-    <row r="1048493" ht="12.8"/>
-    <row r="1048494" ht="12.8"/>
-    <row r="1048495" ht="12.8"/>
-    <row r="1048496" ht="12.8"/>
-    <row r="1048497" ht="12.8"/>
-    <row r="1048498" ht="12.8"/>
-    <row r="1048499" ht="12.8"/>
-    <row r="1048500" ht="12.8"/>
-    <row r="1048501" ht="12.8"/>
-    <row r="1048502" ht="12.8"/>
-    <row r="1048503" ht="12.8"/>
-    <row r="1048504" ht="12.8"/>
-    <row r="1048505" ht="12.8"/>
-    <row r="1048506" ht="12.8"/>
-    <row r="1048507" ht="12.8"/>
-    <row r="1048508" ht="12.8"/>
-    <row r="1048509" ht="12.8"/>
-    <row r="1048510" ht="12.8"/>
-    <row r="1048511" ht="12.8"/>
-    <row r="1048512" ht="12.8"/>
-    <row r="1048513" ht="12.8"/>
-    <row r="1048514" ht="12.8"/>
-    <row r="1048515" ht="12.8"/>
-    <row r="1048516" ht="12.8"/>
-    <row r="1048517" ht="12.8"/>
-    <row r="1048518" ht="12.8"/>
-    <row r="1048519" ht="12.8"/>
-    <row r="1048520" ht="12.8"/>
-    <row r="1048521" ht="12.8"/>
-    <row r="1048522" ht="12.8"/>
-    <row r="1048523" ht="12.8"/>
-    <row r="1048524" ht="12.8"/>
-    <row r="1048525" ht="12.8"/>
-    <row r="1048526" ht="12.8"/>
-    <row r="1048527" ht="12.8"/>
-    <row r="1048528" ht="12.8"/>
-    <row r="1048529" ht="12.8"/>
-    <row r="1048530" ht="12.8"/>
-    <row r="1048531" ht="12.8"/>
-    <row r="1048532" ht="12.8"/>
-    <row r="1048533" ht="12.8"/>
-    <row r="1048534" ht="12.8"/>
-    <row r="1048535" ht="12.8"/>
-    <row r="1048536" ht="12.8"/>
-    <row r="1048537" ht="12.8"/>
-    <row r="1048538" ht="12.8"/>
-    <row r="1048539" ht="12.8"/>
-    <row r="1048540" ht="12.8"/>
-    <row r="1048541" ht="12.8"/>
-    <row r="1048542" ht="12.8"/>
-    <row r="1048543" ht="12.8"/>
-    <row r="1048544" ht="12.8"/>
-    <row r="1048545" ht="12.8"/>
-    <row r="1048546" ht="12.8"/>
-    <row r="1048547" ht="12.8"/>
-    <row r="1048548" ht="12.8"/>
-    <row r="1048549" ht="12.8"/>
-    <row r="1048550" ht="12.8"/>
-    <row r="1048551" ht="12.8"/>
-    <row r="1048552" ht="12.8"/>
-    <row r="1048553" ht="12.8"/>
-    <row r="1048554" ht="12.8"/>
-    <row r="1048555" ht="12.8"/>
+    <row r="1048493" ht="12.8" customHeight="true"/>
+    <row r="1048494" ht="12.8" customHeight="true"/>
+    <row r="1048495" ht="12.8" customHeight="true"/>
+    <row r="1048508" ht="12.8" customHeight="true"/>
+    <row r="1048509" ht="12.8" customHeight="true"/>
+    <row r="1048510" ht="12.8" customHeight="true"/>
+    <row r="1048511" ht="12.8" customHeight="true"/>
+    <row r="1048512" ht="12.8" customHeight="true"/>
+    <row r="1048513" ht="12.8" customHeight="true"/>
+    <row r="1048514" ht="12.8" customHeight="true"/>
+    <row r="1048515" ht="12.8" customHeight="true"/>
+    <row r="1048516" ht="12.8" customHeight="true"/>
+    <row r="1048517" ht="12.8" customHeight="true"/>
+    <row r="1048518" ht="12.8" customHeight="true"/>
+    <row r="1048519" ht="12.8" customHeight="true"/>
+    <row r="1048520" ht="12.8" customHeight="true"/>
+    <row r="1048521" ht="12.8" customHeight="true"/>
+    <row r="1048522" ht="12.8" customHeight="true"/>
+    <row r="1048523" ht="12.8" customHeight="true"/>
+    <row r="1048524" ht="12.8" customHeight="true"/>
+    <row r="1048525" ht="12.8" customHeight="true"/>
+    <row r="1048526" ht="12.8" customHeight="true"/>
+    <row r="1048527" ht="12.8" customHeight="true"/>
+    <row r="1048528" ht="12.8" customHeight="true"/>
+    <row r="1048529" ht="12.8" customHeight="true"/>
+    <row r="1048530" ht="12.8" customHeight="true"/>
+    <row r="1048531" ht="12.8" customHeight="true"/>
+    <row r="1048532" ht="12.8" customHeight="true"/>
+    <row r="1048533" ht="12.8" customHeight="true"/>
+    <row r="1048534" ht="12.8" customHeight="true"/>
+    <row r="1048535" ht="12.8" customHeight="true"/>
+    <row r="1048536" ht="12.8" customHeight="true"/>
+    <row r="1048537" ht="12.8" customHeight="true"/>
+    <row r="1048538" ht="12.8" customHeight="true"/>
+    <row r="1048539" ht="12.8" customHeight="true"/>
+    <row r="1048540" ht="12.8" customHeight="true"/>
+    <row r="1048541" ht="12.8" customHeight="true"/>
+    <row r="1048542" ht="12.8" customHeight="true"/>
+    <row r="1048543" ht="12.8" customHeight="true"/>
+    <row r="1048544" ht="12.8" customHeight="true"/>
+    <row r="1048545" ht="12.8" customHeight="true"/>
+    <row r="1048546" ht="12.8" customHeight="true"/>
+    <row r="1048547" ht="12.8" customHeight="true"/>
+    <row r="1048548" ht="12.8" customHeight="true"/>
+    <row r="1048549" ht="12.8" customHeight="true"/>
+    <row r="1048550" ht="12.8" customHeight="true"/>
+    <row r="1048551" ht="12.8" customHeight="true"/>
+    <row r="1048552" ht="12.8" customHeight="true"/>
+    <row r="1048553" ht="12.8" customHeight="true"/>
+    <row r="1048554" ht="12.8" customHeight="true"/>
+    <row r="1048555" ht="12.8" customHeight="true"/>
+    <row r="1048556" ht="12.8" customHeight="true"/>
+    <row r="1048557" ht="12.8" customHeight="true"/>
+    <row r="1048558" ht="12.8" customHeight="true"/>
+    <row r="1048559" ht="12.8" customHeight="true"/>
+    <row r="1048560" ht="12.8" customHeight="true"/>
+    <row r="1048561" ht="12.8" customHeight="true"/>
     <row r="1048562" ht="12.8" customHeight="true"/>
     <row r="1048563" ht="12.8" customHeight="true"/>
     <row r="1048564" ht="12.8" customHeight="true"/>

</xml_diff>